<commit_message>
Sync laminas_provinciales, dependencia, envejecimiento y otras_relaciones
</commit_message>
<xml_diff>
--- a/output/graficos_dependencia/plot_regional_d_deptot_a_2018_antofagasta.xlsx
+++ b/output/graficos_dependencia/plot_regional_d_deptot_a_2018_antofagasta.xlsx
@@ -1,48 +1,139 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="resumen" sheetId="1" r:id="rId1"/>
-    <sheet name="serie_anual" sheetId="2" r:id="rId2"/>
-    <sheet name="provincias" sheetId="3" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Serie_anual" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Provincias" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Provincias'!$A$1:$C$4</definedName>
+  </definedNames>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t xml:space="preserve">Territorio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nacional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reg_Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reg_Hombres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reg_Mujeres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antofagasta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de creación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-27 19:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIT - MDSF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagen asociada</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidad territorial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Region</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name_prov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Loa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tocopilla</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
       <b/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00135A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,21 +141,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -114,10 +221,6 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -143,15 +246,12 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -177,6 +277,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -352,235 +453,298 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="13.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="13.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="13.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Territorio</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Anio</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Reg_Total</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Reg_Hombres</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Reg_Mujeres</t>
-        </is>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Antofagasta</t>
-        </is>
-      </c>
-      <c r="B2">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="n">
         <v>2018</v>
       </c>
-      <c r="C2">
-        <v>57.05862520210228</v>
-      </c>
-      <c r="D2">
-        <v>50.28564216502235</v>
-      </c>
-      <c r="E2">
-        <v>48.93500276714804</v>
-      </c>
-      <c r="F2">
-        <v>51.65498124898092</v>
+      <c r="C2" s="2" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>50.29</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>48.94</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>51.65</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="24.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="60.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>2018</v>
-      </c>
-      <c r="B2">
-        <v>57.05862520210228</v>
-      </c>
-      <c r="C2">
-        <v>50.28564216502235</v>
+      <c r="A2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>2019</v>
-      </c>
-      <c r="B3">
-        <v>57.69266621582525</v>
-      </c>
-      <c r="C3">
-        <v>50.3171613877681</v>
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>2020</v>
-      </c>
-      <c r="B4">
-        <v>57.63072289364759</v>
-      </c>
-      <c r="C4">
-        <v>49.55453917721474</v>
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <v>2021</v>
-      </c>
-      <c r="B5">
-        <v>58.63423909225823</v>
-      </c>
-      <c r="C5">
-        <v>49.5831380635486</v>
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <v>2022</v>
-      </c>
-      <c r="B6">
-        <v>58.64905447909768</v>
-      </c>
-      <c r="C6">
-        <v>50.77377159302398</v>
+      <c r="A6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <v>2023</v>
-      </c>
-      <c r="B7">
-        <v>59.45184748536308</v>
-      </c>
-      <c r="C7">
-        <v>51.08880227148268</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>2024</v>
-      </c>
-      <c r="B8">
-        <v>59.86337263328625</v>
-      </c>
-      <c r="C8">
-        <v>51.11639849523905</v>
+      <c r="A7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>name_prov</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Ratio</t>
-        </is>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Antofagasta</t>
-        </is>
-      </c>
-      <c r="B2">
+      <c r="A2" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>50.29</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>57.69</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>50.32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>57.63</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>49.55</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>58.63</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>49.58</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>58.65</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>50.77</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>59.45</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>51.09</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>59.86</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>51.12</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C8"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="13.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C2">
-        <v>49.75613833607117</v>
+      <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>49.76</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>El Loa</t>
-        </is>
-      </c>
-      <c r="B3">
+      <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="C3">
-        <v>49.98155484626366</v>
+      <c r="C3" s="2" t="n">
+        <v>49.98</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Tocopilla</t>
-        </is>
-      </c>
-      <c r="B4">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="C4">
-        <v>59.42931128927842</v>
+      <c r="C4" s="2" t="n">
+        <v>59.43</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>